<commit_message>
Changed the buttons and added loading and completed states(indication)
</commit_message>
<xml_diff>
--- a/samples/trial-balance/TB-Annual-2024-25.xlsx
+++ b/samples/trial-balance/TB-Annual-2024-25.xlsx
@@ -1,10 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E73350C-87AE-46F0-96D0-DE7540DBE349}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Trial Balance" state="visible" r:id="rId4"/>
+    <sheet name="Trial Balance" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -79,20 +83,20 @@
     <t>Equity Share Capital</t>
   </si>
   <si>
-    <t>Other Equity</t>
+    <t>Unknown</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -455,11 +459,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -470,7 +474,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -481,7 +485,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -492,7 +496,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -503,7 +507,7 @@
         <v>25000</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -514,7 +518,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -525,7 +529,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -536,7 +540,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -547,7 +551,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -558,7 +562,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -569,7 +573,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>13</v>
       </c>
@@ -580,7 +584,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>14</v>
       </c>
@@ -591,7 +595,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>15</v>
       </c>
@@ -602,7 +606,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>16</v>
       </c>
@@ -613,7 +617,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>17</v>
       </c>
@@ -624,7 +628,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>18</v>
       </c>
@@ -635,7 +639,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>19</v>
       </c>
@@ -646,7 +650,7 @@
         <v>45000</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -657,7 +661,7 @@
         <v>25000</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>21</v>
       </c>
@@ -668,7 +672,7 @@
         <v>100000</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>22</v>
       </c>
@@ -681,6 +685,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>